<commit_message>
ability to add qgisand attaching scans
</commit_message>
<xml_diff>
--- a/xlsforms/dqa_form.xlsx
+++ b/xlsforms/dqa_form.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -770,28 +770,164 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>geopoint</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>submitted_by</t>
+          <t>location</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Submitted by (your name)</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
+          <t>Location of this activity</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Record the GPS location while you are at the facility.</t>
+        </is>
+      </c>
       <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>photo_1</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Photo 1 of this activity</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>photo_2</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Photo 2 of this activity</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>photo_3</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Photo 3 of this activity</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>attendance_photo</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Attendance list - photo</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>attendance_file</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Attendance list - file (PDF or Excel)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>submitted_by</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Submitted by (your name)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>